<commit_message>
Add automation scripts for crypto and news sentiment
</commit_message>
<xml_diff>
--- a/crypto_report.xlsx
+++ b/crypto_report.xlsx
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-05 17:19:53</t>
+          <t>2026-05-05 22:01:50</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>631.3200000000001</v>
+        <v>631.78</v>
       </c>
       <c r="D2" t="n">
-        <v>0.64</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-05 17:19:53</t>
+          <t>2026-05-05 22:01:50</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -468,16 +468,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>81555</v>
+        <v>81623</v>
       </c>
       <c r="D3" t="n">
-        <v>1.89</v>
+        <v>2.07</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-05 17:19:53</t>
+          <t>2026-05-05 22:01:50</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -486,10 +486,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2381.5</v>
+        <v>2372.07</v>
       </c>
       <c r="D4" t="n">
-        <v>0.72</v>
+        <v>0.76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>